<commit_message>
Expand benchmark: weighted metrics, location-aware failures, summary Excel
- Add 4 quizzes + 6 tests schema (quiz_weight=5%, test_weight=80/6%)
- Add percentile rank, per-student z-score, per-assessment z-scores
- Expand test inputs to 25 students (40 for 05_large) with new columns
- Regenerate all ground truth JSONs with new metric structure
- Add exact Excel cell location (sheet, row, column_letter) to every failure
- Add failures_by_location grouping and error_pattern_summary with root_cause_hypotheses
- Add generate_summary_excel() producing color-coded benchmark_summary.xlsx
- Add generate_inputs.py for reproducible CSV generation
- Include all v0 eval results and generated Excel outputs

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/v0/03_ties_output.xlsx
+++ b/outputs/v0/03_ties_output.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Student Stats" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Stats" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overall" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessment Stats" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Z-Scores" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overall" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:V26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,65 +427,105 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>test1</t>
+          <t>quiz_1</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>test2</t>
+          <t>quiz_2</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>test3</t>
+          <t>quiz_3</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>test4</t>
+          <t>quiz_4</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>test5</t>
+          <t>test_1</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>average</t>
+          <t>test_2</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>test_3</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>test_4</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>test_5</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>test_6</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>simple_average</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>weighted_average</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>letter_grade</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>slope</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>std_dev</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>highest_score</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>lowest_score</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>rank</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>percentile</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>z_score</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
         <is>
           <t>above_class_average</t>
         </is>
@@ -497,44 +538,68 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C2" t="n">
         <v>82</v>
       </c>
       <c r="D2" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E2" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G2" t="n">
-        <v>81</v>
-      </c>
-      <c r="H2" t="inlineStr">
+        <v>82</v>
+      </c>
+      <c r="H2" t="n">
+        <v>82</v>
+      </c>
+      <c r="I2" t="n">
+        <v>82</v>
+      </c>
+      <c r="J2" t="n">
+        <v>82</v>
+      </c>
+      <c r="K2" t="n">
+        <v>82</v>
+      </c>
+      <c r="L2" t="n">
+        <v>82</v>
+      </c>
+      <c r="M2" t="n">
+        <v>82</v>
+      </c>
+      <c r="N2" t="inlineStr">
         <is>
           <t>B-</t>
         </is>
       </c>
-      <c r="I2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1.581139</v>
-      </c>
-      <c r="K2" t="n">
-        <v>83</v>
-      </c>
-      <c r="L2" t="n">
-        <v>79</v>
-      </c>
-      <c r="M2" t="n">
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>82</v>
+      </c>
+      <c r="R2" t="n">
+        <v>82</v>
+      </c>
+      <c r="S2" t="n">
         <v>2</v>
       </c>
-      <c r="N2" t="b">
+      <c r="T2" t="n">
+        <v>83.333333</v>
+      </c>
+      <c r="U2" t="n">
+        <v>1.118892</v>
+      </c>
+      <c r="V2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -545,44 +610,68 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C3" t="n">
         <v>82</v>
       </c>
       <c r="D3" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E3" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F3" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G3" t="n">
-        <v>81</v>
-      </c>
-      <c r="H3" t="inlineStr">
+        <v>82</v>
+      </c>
+      <c r="H3" t="n">
+        <v>82</v>
+      </c>
+      <c r="I3" t="n">
+        <v>82</v>
+      </c>
+      <c r="J3" t="n">
+        <v>82</v>
+      </c>
+      <c r="K3" t="n">
+        <v>82</v>
+      </c>
+      <c r="L3" t="n">
+        <v>82</v>
+      </c>
+      <c r="M3" t="n">
+        <v>82</v>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>B-</t>
         </is>
       </c>
-      <c r="I3" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J3" t="n">
-        <v>1.581139</v>
-      </c>
-      <c r="K3" t="n">
-        <v>83</v>
-      </c>
-      <c r="L3" t="n">
-        <v>79</v>
-      </c>
-      <c r="M3" t="n">
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>82</v>
+      </c>
+      <c r="R3" t="n">
+        <v>82</v>
+      </c>
+      <c r="S3" t="n">
         <v>2</v>
       </c>
-      <c r="N3" t="b">
+      <c r="T3" t="n">
+        <v>83.333333</v>
+      </c>
+      <c r="U3" t="n">
+        <v>1.118892</v>
+      </c>
+      <c r="V3" t="b">
         <v>1</v>
       </c>
     </row>
@@ -593,45 +682,69 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C4" t="n">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="D4" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="E4" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="F4" t="n">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G4" t="n">
-        <v>75</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+        <v>82</v>
+      </c>
+      <c r="H4" t="n">
+        <v>82</v>
       </c>
       <c r="I4" t="n">
-        <v>0.3</v>
+        <v>82</v>
       </c>
       <c r="J4" t="n">
-        <v>1.581139</v>
+        <v>82</v>
       </c>
       <c r="K4" t="n">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="L4" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="M4" t="n">
-        <v>4</v>
-      </c>
-      <c r="N4" t="b">
-        <v>0</v>
+        <v>82</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>82</v>
+      </c>
+      <c r="R4" t="n">
+        <v>82</v>
+      </c>
+      <c r="S4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T4" t="n">
+        <v>83.333333</v>
+      </c>
+      <c r="U4" t="n">
+        <v>1.118892</v>
+      </c>
+      <c r="V4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -641,45 +754,69 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="C5" t="n">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D5" t="n">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="E5" t="n">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="F5" t="n">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="G5" t="n">
-        <v>90</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>A-</t>
-        </is>
+        <v>75</v>
+      </c>
+      <c r="H5" t="n">
+        <v>75</v>
       </c>
       <c r="I5" t="n">
-        <v>0.5</v>
+        <v>75</v>
       </c>
       <c r="J5" t="n">
-        <v>1.581139</v>
+        <v>75</v>
       </c>
       <c r="K5" t="n">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="L5" t="n">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="M5" t="n">
-        <v>1</v>
-      </c>
-      <c r="N5" t="b">
-        <v>1</v>
+        <v>75</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>75</v>
+      </c>
+      <c r="R5" t="n">
+        <v>75</v>
+      </c>
+      <c r="S5" t="n">
+        <v>7</v>
+      </c>
+      <c r="T5" t="n">
+        <v>54.166667</v>
+      </c>
+      <c r="U5" t="n">
+        <v>-0.06961199999999999</v>
+      </c>
+      <c r="V5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -692,41 +829,1505 @@
         <v>75</v>
       </c>
       <c r="C6" t="n">
+        <v>75</v>
+      </c>
+      <c r="D6" t="n">
+        <v>75</v>
+      </c>
+      <c r="E6" t="n">
+        <v>75</v>
+      </c>
+      <c r="F6" t="n">
+        <v>75</v>
+      </c>
+      <c r="G6" t="n">
+        <v>75</v>
+      </c>
+      <c r="H6" t="n">
+        <v>75</v>
+      </c>
+      <c r="I6" t="n">
+        <v>75</v>
+      </c>
+      <c r="J6" t="n">
+        <v>75</v>
+      </c>
+      <c r="K6" t="n">
+        <v>75</v>
+      </c>
+      <c r="L6" t="n">
+        <v>75</v>
+      </c>
+      <c r="M6" t="n">
+        <v>75</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>75</v>
+      </c>
+      <c r="R6" t="n">
+        <v>75</v>
+      </c>
+      <c r="S6" t="n">
+        <v>7</v>
+      </c>
+      <c r="T6" t="n">
+        <v>54.166667</v>
+      </c>
+      <c r="U6" t="n">
+        <v>-0.06961199999999999</v>
+      </c>
+      <c r="V6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>S006</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>75</v>
+      </c>
+      <c r="C7" t="n">
+        <v>75</v>
+      </c>
+      <c r="D7" t="n">
+        <v>75</v>
+      </c>
+      <c r="E7" t="n">
+        <v>75</v>
+      </c>
+      <c r="F7" t="n">
+        <v>75</v>
+      </c>
+      <c r="G7" t="n">
+        <v>75</v>
+      </c>
+      <c r="H7" t="n">
+        <v>75</v>
+      </c>
+      <c r="I7" t="n">
+        <v>75</v>
+      </c>
+      <c r="J7" t="n">
+        <v>75</v>
+      </c>
+      <c r="K7" t="n">
+        <v>75</v>
+      </c>
+      <c r="L7" t="n">
+        <v>75</v>
+      </c>
+      <c r="M7" t="n">
+        <v>75</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>75</v>
+      </c>
+      <c r="R7" t="n">
+        <v>75</v>
+      </c>
+      <c r="S7" t="n">
+        <v>7</v>
+      </c>
+      <c r="T7" t="n">
+        <v>54.166667</v>
+      </c>
+      <c r="U7" t="n">
+        <v>-0.06961199999999999</v>
+      </c>
+      <c r="V7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>S007</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>90</v>
+      </c>
+      <c r="C8" t="n">
+        <v>90</v>
+      </c>
+      <c r="D8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E8" t="n">
+        <v>90</v>
+      </c>
+      <c r="F8" t="n">
+        <v>90</v>
+      </c>
+      <c r="G8" t="n">
+        <v>90</v>
+      </c>
+      <c r="H8" t="n">
+        <v>90</v>
+      </c>
+      <c r="I8" t="n">
+        <v>90</v>
+      </c>
+      <c r="J8" t="n">
+        <v>90</v>
+      </c>
+      <c r="K8" t="n">
+        <v>90</v>
+      </c>
+      <c r="L8" t="n">
+        <v>90</v>
+      </c>
+      <c r="M8" t="n">
+        <v>90</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>90</v>
+      </c>
+      <c r="R8" t="n">
+        <v>90</v>
+      </c>
+      <c r="S8" t="n">
+        <v>1</v>
+      </c>
+      <c r="T8" t="n">
+        <v>95.833333</v>
+      </c>
+      <c r="U8" t="n">
+        <v>2.477184</v>
+      </c>
+      <c r="V8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>S008</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>90</v>
+      </c>
+      <c r="C9" t="n">
+        <v>90</v>
+      </c>
+      <c r="D9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E9" t="n">
+        <v>90</v>
+      </c>
+      <c r="F9" t="n">
+        <v>90</v>
+      </c>
+      <c r="G9" t="n">
+        <v>90</v>
+      </c>
+      <c r="H9" t="n">
+        <v>90</v>
+      </c>
+      <c r="I9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J9" t="n">
+        <v>90</v>
+      </c>
+      <c r="K9" t="n">
+        <v>90</v>
+      </c>
+      <c r="L9" t="n">
+        <v>90</v>
+      </c>
+      <c r="M9" t="n">
+        <v>90</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>90</v>
+      </c>
+      <c r="R9" t="n">
+        <v>90</v>
+      </c>
+      <c r="S9" t="n">
+        <v>1</v>
+      </c>
+      <c r="T9" t="n">
+        <v>95.833333</v>
+      </c>
+      <c r="U9" t="n">
+        <v>2.477184</v>
+      </c>
+      <c r="V9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>S009</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>68</v>
+      </c>
+      <c r="C10" t="n">
+        <v>68</v>
+      </c>
+      <c r="D10" t="n">
+        <v>68</v>
+      </c>
+      <c r="E10" t="n">
+        <v>68</v>
+      </c>
+      <c r="F10" t="n">
+        <v>68</v>
+      </c>
+      <c r="G10" t="n">
+        <v>68</v>
+      </c>
+      <c r="H10" t="n">
+        <v>68</v>
+      </c>
+      <c r="I10" t="n">
+        <v>68</v>
+      </c>
+      <c r="J10" t="n">
+        <v>68</v>
+      </c>
+      <c r="K10" t="n">
+        <v>68</v>
+      </c>
+      <c r="L10" t="n">
+        <v>68</v>
+      </c>
+      <c r="M10" t="n">
+        <v>68</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>D+</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>68</v>
+      </c>
+      <c r="R10" t="n">
+        <v>68</v>
+      </c>
+      <c r="S10" t="n">
+        <v>18</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" t="n">
+        <v>-1.258117</v>
+      </c>
+      <c r="V10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>S010</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>68</v>
+      </c>
+      <c r="C11" t="n">
+        <v>68</v>
+      </c>
+      <c r="D11" t="n">
+        <v>68</v>
+      </c>
+      <c r="E11" t="n">
+        <v>68</v>
+      </c>
+      <c r="F11" t="n">
+        <v>68</v>
+      </c>
+      <c r="G11" t="n">
+        <v>68</v>
+      </c>
+      <c r="H11" t="n">
+        <v>68</v>
+      </c>
+      <c r="I11" t="n">
+        <v>68</v>
+      </c>
+      <c r="J11" t="n">
+        <v>68</v>
+      </c>
+      <c r="K11" t="n">
+        <v>68</v>
+      </c>
+      <c r="L11" t="n">
+        <v>68</v>
+      </c>
+      <c r="M11" t="n">
+        <v>68</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>D+</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>68</v>
+      </c>
+      <c r="R11" t="n">
+        <v>68</v>
+      </c>
+      <c r="S11" t="n">
+        <v>18</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" t="n">
+        <v>-1.258117</v>
+      </c>
+      <c r="V11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>S011</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>68</v>
+      </c>
+      <c r="C12" t="n">
+        <v>68</v>
+      </c>
+      <c r="D12" t="n">
+        <v>68</v>
+      </c>
+      <c r="E12" t="n">
+        <v>68</v>
+      </c>
+      <c r="F12" t="n">
+        <v>68</v>
+      </c>
+      <c r="G12" t="n">
+        <v>68</v>
+      </c>
+      <c r="H12" t="n">
+        <v>68</v>
+      </c>
+      <c r="I12" t="n">
+        <v>68</v>
+      </c>
+      <c r="J12" t="n">
+        <v>68</v>
+      </c>
+      <c r="K12" t="n">
+        <v>68</v>
+      </c>
+      <c r="L12" t="n">
+        <v>68</v>
+      </c>
+      <c r="M12" t="n">
+        <v>68</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>D+</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>68</v>
+      </c>
+      <c r="R12" t="n">
+        <v>68</v>
+      </c>
+      <c r="S12" t="n">
+        <v>18</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" t="n">
+        <v>-1.258117</v>
+      </c>
+      <c r="V12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>S012</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>67</v>
+      </c>
+      <c r="C13" t="n">
+        <v>71</v>
+      </c>
+      <c r="D13" t="n">
+        <v>66</v>
+      </c>
+      <c r="E13" t="n">
+        <v>77</v>
+      </c>
+      <c r="F13" t="n">
+        <v>66</v>
+      </c>
+      <c r="G13" t="n">
+        <v>89</v>
+      </c>
+      <c r="H13" t="n">
+        <v>63</v>
+      </c>
+      <c r="I13" t="n">
+        <v>63</v>
+      </c>
+      <c r="J13" t="n">
+        <v>60</v>
+      </c>
+      <c r="K13" t="n">
+        <v>77</v>
+      </c>
+      <c r="L13" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="M13" t="n">
+        <v>69.783333</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>C-</t>
+        </is>
+      </c>
+      <c r="O13" t="n">
+        <v>-0.127273</v>
+      </c>
+      <c r="P13" t="n">
+        <v>8.812239</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>89</v>
+      </c>
+      <c r="R13" t="n">
+        <v>60</v>
+      </c>
+      <c r="S13" t="n">
+        <v>16</v>
+      </c>
+      <c r="T13" t="n">
+        <v>16.666667</v>
+      </c>
+      <c r="U13" t="n">
+        <v>-0.955332</v>
+      </c>
+      <c r="V13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>S013</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>63</v>
+      </c>
+      <c r="C14" t="n">
+        <v>86</v>
+      </c>
+      <c r="D14" t="n">
+        <v>67</v>
+      </c>
+      <c r="E14" t="n">
+        <v>82</v>
+      </c>
+      <c r="F14" t="n">
+        <v>92</v>
+      </c>
+      <c r="G14" t="n">
+        <v>65</v>
+      </c>
+      <c r="H14" t="n">
+        <v>50</v>
+      </c>
+      <c r="I14" t="n">
+        <v>79</v>
+      </c>
+      <c r="J14" t="n">
+        <v>79</v>
+      </c>
+      <c r="K14" t="n">
+        <v>72</v>
+      </c>
+      <c r="L14" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="M14" t="n">
+        <v>73.166667</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O14" t="n">
+        <v>-0.187879</v>
+      </c>
+      <c r="P14" t="n">
+        <v>12.518875</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>92</v>
+      </c>
+      <c r="R14" t="n">
+        <v>50</v>
+      </c>
+      <c r="S14" t="n">
+        <v>13</v>
+      </c>
+      <c r="T14" t="n">
+        <v>29.166667</v>
+      </c>
+      <c r="U14" t="n">
+        <v>-0.380887</v>
+      </c>
+      <c r="V14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>S014</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>75</v>
+      </c>
+      <c r="C15" t="n">
+        <v>87</v>
+      </c>
+      <c r="D15" t="n">
+        <v>59</v>
+      </c>
+      <c r="E15" t="n">
+        <v>75</v>
+      </c>
+      <c r="F15" t="n">
+        <v>91</v>
+      </c>
+      <c r="G15" t="n">
+        <v>67</v>
+      </c>
+      <c r="H15" t="n">
+        <v>72</v>
+      </c>
+      <c r="I15" t="n">
+        <v>72</v>
+      </c>
+      <c r="J15" t="n">
+        <v>84</v>
+      </c>
+      <c r="K15" t="n">
+        <v>57</v>
+      </c>
+      <c r="L15" t="n">
+        <v>73.90000000000001</v>
+      </c>
+      <c r="M15" t="n">
+        <v>73.86666700000001</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O15" t="n">
+        <v>-0.915152</v>
+      </c>
+      <c r="P15" t="n">
+        <v>11.209619</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>91</v>
+      </c>
+      <c r="R15" t="n">
+        <v>57</v>
+      </c>
+      <c r="S15" t="n">
+        <v>10</v>
+      </c>
+      <c r="T15" t="n">
+        <v>41.666667</v>
+      </c>
+      <c r="U15" t="n">
+        <v>-0.262037</v>
+      </c>
+      <c r="V15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>S015</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>71</v>
+      </c>
+      <c r="C16" t="n">
+        <v>84</v>
+      </c>
+      <c r="D16" t="n">
+        <v>88</v>
+      </c>
+      <c r="E16" t="n">
+        <v>64</v>
+      </c>
+      <c r="F16" t="n">
+        <v>78</v>
+      </c>
+      <c r="G16" t="n">
+        <v>71</v>
+      </c>
+      <c r="H16" t="n">
+        <v>77</v>
+      </c>
+      <c r="I16" t="n">
+        <v>88</v>
+      </c>
+      <c r="J16" t="n">
+        <v>58</v>
+      </c>
+      <c r="K16" t="n">
+        <v>65</v>
+      </c>
+      <c r="L16" t="n">
+        <v>74.40000000000001</v>
+      </c>
+      <c r="M16" t="n">
+        <v>73.61666700000001</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>-1.236364</v>
+      </c>
+      <c r="P16" t="n">
+        <v>10.383748</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>88</v>
+      </c>
+      <c r="R16" t="n">
+        <v>58</v>
+      </c>
+      <c r="S16" t="n">
+        <v>11</v>
+      </c>
+      <c r="T16" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="U16" t="n">
+        <v>-0.304484</v>
+      </c>
+      <c r="V16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>S016</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>72</v>
+      </c>
+      <c r="C17" t="n">
+        <v>54</v>
+      </c>
+      <c r="D17" t="n">
+        <v>58</v>
+      </c>
+      <c r="E17" t="n">
+        <v>73</v>
+      </c>
+      <c r="F17" t="n">
+        <v>79</v>
+      </c>
+      <c r="G17" t="n">
+        <v>75</v>
+      </c>
+      <c r="H17" t="n">
+        <v>68</v>
+      </c>
+      <c r="I17" t="n">
+        <v>73</v>
+      </c>
+      <c r="J17" t="n">
+        <v>78</v>
+      </c>
+      <c r="K17" t="n">
+        <v>77</v>
+      </c>
+      <c r="L17" t="n">
+        <v>70.7</v>
+      </c>
+      <c r="M17" t="n">
+        <v>72.84999999999999</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>1.630303</v>
+      </c>
+      <c r="P17" t="n">
+        <v>8.433399</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>79</v>
+      </c>
+      <c r="R17" t="n">
+        <v>54</v>
+      </c>
+      <c r="S17" t="n">
+        <v>15</v>
+      </c>
+      <c r="T17" t="n">
+        <v>20.833333</v>
+      </c>
+      <c r="U17" t="n">
+        <v>-0.434653</v>
+      </c>
+      <c r="V17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>S017</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>61</v>
+      </c>
+      <c r="C18" t="n">
+        <v>60</v>
+      </c>
+      <c r="D18" t="n">
+        <v>84</v>
+      </c>
+      <c r="E18" t="n">
+        <v>58</v>
+      </c>
+      <c r="F18" t="n">
+        <v>82</v>
+      </c>
+      <c r="G18" t="n">
+        <v>80</v>
+      </c>
+      <c r="H18" t="n">
+        <v>66</v>
+      </c>
+      <c r="I18" t="n">
         <v>74</v>
       </c>
-      <c r="D6" t="n">
+      <c r="J18" t="n">
+        <v>80</v>
+      </c>
+      <c r="K18" t="n">
+        <v>69</v>
+      </c>
+      <c r="L18" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="M18" t="n">
+        <v>73.283333</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O18" t="n">
+        <v>1.115152</v>
+      </c>
+      <c r="P18" t="n">
+        <v>9.879270999999999</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>84</v>
+      </c>
+      <c r="R18" t="n">
+        <v>58</v>
+      </c>
+      <c r="S18" t="n">
+        <v>12</v>
+      </c>
+      <c r="T18" t="n">
+        <v>33.333333</v>
+      </c>
+      <c r="U18" t="n">
+        <v>-0.361079</v>
+      </c>
+      <c r="V18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>S018</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>67</v>
+      </c>
+      <c r="C19" t="n">
+        <v>82</v>
+      </c>
+      <c r="D19" t="n">
+        <v>81</v>
+      </c>
+      <c r="E19" t="n">
+        <v>86</v>
+      </c>
+      <c r="F19" t="n">
+        <v>63</v>
+      </c>
+      <c r="G19" t="n">
         <v>76</v>
       </c>
-      <c r="E6" t="n">
+      <c r="H19" t="n">
         <v>73</v>
       </c>
-      <c r="F6" t="n">
+      <c r="I19" t="n">
+        <v>83</v>
+      </c>
+      <c r="J19" t="n">
+        <v>70</v>
+      </c>
+      <c r="K19" t="n">
+        <v>63</v>
+      </c>
+      <c r="L19" t="n">
+        <v>74.40000000000001</v>
+      </c>
+      <c r="M19" t="n">
+        <v>72.86666700000001</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O19" t="n">
+        <v>-0.824242</v>
+      </c>
+      <c r="P19" t="n">
+        <v>8.4879</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>86</v>
+      </c>
+      <c r="R19" t="n">
+        <v>63</v>
+      </c>
+      <c r="S19" t="n">
+        <v>14</v>
+      </c>
+      <c r="T19" t="n">
+        <v>25</v>
+      </c>
+      <c r="U19" t="n">
+        <v>-0.431823</v>
+      </c>
+      <c r="V19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>S019</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>78</v>
+      </c>
+      <c r="C20" t="n">
+        <v>58</v>
+      </c>
+      <c r="D20" t="n">
+        <v>65</v>
+      </c>
+      <c r="E20" t="n">
+        <v>73</v>
+      </c>
+      <c r="F20" t="n">
+        <v>85</v>
+      </c>
+      <c r="G20" t="n">
+        <v>59</v>
+      </c>
+      <c r="H20" t="n">
+        <v>68</v>
+      </c>
+      <c r="I20" t="n">
+        <v>69</v>
+      </c>
+      <c r="J20" t="n">
+        <v>53</v>
+      </c>
+      <c r="K20" t="n">
         <v>77</v>
       </c>
-      <c r="G6" t="n">
-        <v>75</v>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="L20" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="M20" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>D+</t>
+        </is>
+      </c>
+      <c r="O20" t="n">
+        <v>-0.393939</v>
+      </c>
+      <c r="P20" t="n">
+        <v>10.047111</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>85</v>
+      </c>
+      <c r="R20" t="n">
+        <v>53</v>
+      </c>
+      <c r="S20" t="n">
+        <v>17</v>
+      </c>
+      <c r="T20" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="U20" t="n">
+        <v>-1.173224</v>
+      </c>
+      <c r="V20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>S020</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>69</v>
+      </c>
+      <c r="C21" t="n">
+        <v>72</v>
+      </c>
+      <c r="D21" t="n">
+        <v>77</v>
+      </c>
+      <c r="E21" t="n">
+        <v>62</v>
+      </c>
+      <c r="F21" t="n">
+        <v>61</v>
+      </c>
+      <c r="G21" t="n">
+        <v>87</v>
+      </c>
+      <c r="H21" t="n">
+        <v>72</v>
+      </c>
+      <c r="I21" t="n">
+        <v>84</v>
+      </c>
+      <c r="J21" t="n">
+        <v>87</v>
+      </c>
+      <c r="K21" t="n">
+        <v>77</v>
+      </c>
+      <c r="L21" t="n">
+        <v>74.8</v>
+      </c>
+      <c r="M21" t="n">
+        <v>76.40000000000001</v>
+      </c>
+      <c r="N21" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I6" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="J6" t="n">
-        <v>1.581139</v>
-      </c>
-      <c r="K6" t="n">
+      <c r="O21" t="n">
+        <v>1.624242</v>
+      </c>
+      <c r="P21" t="n">
+        <v>9.402127</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>87</v>
+      </c>
+      <c r="R21" t="n">
+        <v>61</v>
+      </c>
+      <c r="S21" t="n">
+        <v>3</v>
+      </c>
+      <c r="T21" t="n">
+        <v>79.166667</v>
+      </c>
+      <c r="U21" t="n">
+        <v>0.168089</v>
+      </c>
+      <c r="V21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>S021</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>65</v>
+      </c>
+      <c r="C22" t="n">
+        <v>93</v>
+      </c>
+      <c r="D22" t="n">
+        <v>72</v>
+      </c>
+      <c r="E22" t="n">
+        <v>69</v>
+      </c>
+      <c r="F22" t="n">
         <v>77</v>
       </c>
-      <c r="L6" t="n">
+      <c r="G22" t="n">
+        <v>82</v>
+      </c>
+      <c r="H22" t="n">
+        <v>78</v>
+      </c>
+      <c r="I22" t="n">
+        <v>69</v>
+      </c>
+      <c r="J22" t="n">
+        <v>82</v>
+      </c>
+      <c r="K22" t="n">
+        <v>66</v>
+      </c>
+      <c r="L22" t="n">
+        <v>75.3</v>
+      </c>
+      <c r="M22" t="n">
+        <v>75.483333</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O22" t="n">
+        <v>-0.309091</v>
+      </c>
+      <c r="P22" t="n">
+        <v>8.794568999999999</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>93</v>
+      </c>
+      <c r="R22" t="n">
+        <v>65</v>
+      </c>
+      <c r="S22" t="n">
+        <v>6</v>
+      </c>
+      <c r="T22" t="n">
+        <v>66.666667</v>
+      </c>
+      <c r="U22" t="n">
+        <v>0.012451</v>
+      </c>
+      <c r="V22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>S022</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>79</v>
+      </c>
+      <c r="C23" t="n">
         <v>73</v>
       </c>
-      <c r="M6" t="n">
+      <c r="D23" t="n">
+        <v>66</v>
+      </c>
+      <c r="E23" t="n">
+        <v>82</v>
+      </c>
+      <c r="F23" t="n">
+        <v>78</v>
+      </c>
+      <c r="G23" t="n">
+        <v>68</v>
+      </c>
+      <c r="H23" t="n">
+        <v>67</v>
+      </c>
+      <c r="I23" t="n">
+        <v>74</v>
+      </c>
+      <c r="J23" t="n">
+        <v>83</v>
+      </c>
+      <c r="K23" t="n">
+        <v>87</v>
+      </c>
+      <c r="L23" t="n">
+        <v>75.7</v>
+      </c>
+      <c r="M23" t="n">
+        <v>75.933333</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O23" t="n">
+        <v>0.769697</v>
+      </c>
+      <c r="P23" t="n">
+        <v>7.273239</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>87</v>
+      </c>
+      <c r="R23" t="n">
+        <v>66</v>
+      </c>
+      <c r="S23" t="n">
         <v>4</v>
       </c>
-      <c r="N6" t="b">
+      <c r="T23" t="n">
+        <v>75</v>
+      </c>
+      <c r="U23" t="n">
+        <v>0.088855</v>
+      </c>
+      <c r="V23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>S023</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>70</v>
+      </c>
+      <c r="C24" t="n">
+        <v>82</v>
+      </c>
+      <c r="D24" t="n">
+        <v>86</v>
+      </c>
+      <c r="E24" t="n">
+        <v>65</v>
+      </c>
+      <c r="F24" t="n">
+        <v>72</v>
+      </c>
+      <c r="G24" t="n">
+        <v>59</v>
+      </c>
+      <c r="H24" t="n">
+        <v>72</v>
+      </c>
+      <c r="I24" t="n">
+        <v>80</v>
+      </c>
+      <c r="J24" t="n">
+        <v>76</v>
+      </c>
+      <c r="K24" t="n">
+        <v>82</v>
+      </c>
+      <c r="L24" t="n">
+        <v>74.40000000000001</v>
+      </c>
+      <c r="M24" t="n">
+        <v>73.95</v>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O24" t="n">
+        <v>0.266667</v>
+      </c>
+      <c r="P24" t="n">
+        <v>8.435375000000001</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>86</v>
+      </c>
+      <c r="R24" t="n">
+        <v>59</v>
+      </c>
+      <c r="S24" t="n">
+        <v>9</v>
+      </c>
+      <c r="T24" t="n">
+        <v>45.833333</v>
+      </c>
+      <c r="U24" t="n">
+        <v>-0.247888</v>
+      </c>
+      <c r="V24" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>S024</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>76</v>
+      </c>
+      <c r="C25" t="n">
+        <v>64</v>
+      </c>
+      <c r="D25" t="n">
+        <v>75</v>
+      </c>
+      <c r="E25" t="n">
+        <v>90</v>
+      </c>
+      <c r="F25" t="n">
+        <v>61</v>
+      </c>
+      <c r="G25" t="n">
+        <v>95</v>
+      </c>
+      <c r="H25" t="n">
+        <v>73</v>
+      </c>
+      <c r="I25" t="n">
+        <v>72</v>
+      </c>
+      <c r="J25" t="n">
+        <v>64</v>
+      </c>
+      <c r="K25" t="n">
+        <v>88</v>
+      </c>
+      <c r="L25" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="M25" t="n">
+        <v>75.65000000000001</v>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O25" t="n">
+        <v>0.460606</v>
+      </c>
+      <c r="P25" t="n">
+        <v>11.735985</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>95</v>
+      </c>
+      <c r="R25" t="n">
+        <v>61</v>
+      </c>
+      <c r="S25" t="n">
+        <v>5</v>
+      </c>
+      <c r="T25" t="n">
+        <v>70.833333</v>
+      </c>
+      <c r="U25" t="n">
+        <v>0.040749</v>
+      </c>
+      <c r="V25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>S025</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>50</v>
+      </c>
+      <c r="C26" t="n">
+        <v>81</v>
+      </c>
+      <c r="D26" t="n">
+        <v>90</v>
+      </c>
+      <c r="E26" t="n">
+        <v>77</v>
+      </c>
+      <c r="F26" t="n">
+        <v>76</v>
+      </c>
+      <c r="G26" t="n">
+        <v>93</v>
+      </c>
+      <c r="H26" t="n">
+        <v>61</v>
+      </c>
+      <c r="I26" t="n">
+        <v>82</v>
+      </c>
+      <c r="J26" t="n">
+        <v>65</v>
+      </c>
+      <c r="K26" t="n">
+        <v>73</v>
+      </c>
+      <c r="L26" t="n">
+        <v>74.8</v>
+      </c>
+      <c r="M26" t="n">
+        <v>74.90000000000001</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O26" t="n">
+        <v>0.145455</v>
+      </c>
+      <c r="P26" t="n">
+        <v>13.180794</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>93</v>
+      </c>
+      <c r="R26" t="n">
+        <v>50</v>
+      </c>
+      <c r="S26" t="n">
+        <v>8</v>
+      </c>
+      <c r="T26" t="n">
+        <v>50</v>
+      </c>
+      <c r="U26" t="n">
+        <v>-0.086591</v>
+      </c>
+      <c r="V26" t="b">
         <v>0</v>
       </c>
     </row>
@@ -741,13 +2342,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>assessment</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -774,96 +2375,191 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>test1</t>
+          <t>quiz_1</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>80</v>
+        <v>72.72</v>
       </c>
       <c r="C2" t="n">
-        <v>6.123724</v>
+        <v>8.942036</v>
       </c>
       <c r="D2" t="n">
         <v>90</v>
       </c>
       <c r="E2" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>test2</t>
+          <t>quiz_2</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>80</v>
+        <v>76.08</v>
       </c>
       <c r="C3" t="n">
-        <v>6</v>
+        <v>10.455939</v>
       </c>
       <c r="D3" t="n">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="E3" t="n">
-        <v>74</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>test3</t>
+          <t>quiz_3</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>80.2</v>
+        <v>75.56</v>
       </c>
       <c r="C4" t="n">
-        <v>6.220932</v>
+        <v>9.687105000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E4" t="n">
-        <v>76</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>test4</t>
+          <t>quiz_4</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>79.40000000000001</v>
+        <v>75.52</v>
       </c>
       <c r="C5" t="n">
-        <v>6.69328</v>
+        <v>8.926178999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E5" t="n">
-        <v>73</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>test5</t>
+          <t>test_1</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>82.40000000000001</v>
+        <v>76.64</v>
       </c>
       <c r="C6" t="n">
-        <v>6.14817</v>
+        <v>9.209958</v>
       </c>
       <c r="D6" t="n">
         <v>92</v>
       </c>
       <c r="E6" t="n">
-        <v>77</v>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>test_2</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>76.84</v>
+      </c>
+      <c r="C7" t="n">
+        <v>10.286237</v>
+      </c>
+      <c r="D7" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>test_3</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>72.59999999999999</v>
+      </c>
+      <c r="C8" t="n">
+        <v>8.793937</v>
+      </c>
+      <c r="D8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E8" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>test_4</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>76.68000000000001</v>
+      </c>
+      <c r="C9" t="n">
+        <v>7.409004</v>
+      </c>
+      <c r="D9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E9" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>test_5</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>74.95999999999999</v>
+      </c>
+      <c r="C10" t="n">
+        <v>9.951884</v>
+      </c>
+      <c r="D10" t="n">
+        <v>90</v>
+      </c>
+      <c r="E10" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>test_6</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>75.40000000000001</v>
+      </c>
+      <c r="C11" t="n">
+        <v>8.698658999999999</v>
+      </c>
+      <c r="D11" t="n">
+        <v>90</v>
+      </c>
+      <c r="E11" t="n">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -877,6 +2573,1002 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>student_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>quiz_1</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>quiz_2</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>quiz_3</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>quiz_4</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>test_1</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>test_2</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>test_3</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>test_4</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>test_5</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>test_6</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1.037795</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.566185</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.664801</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.725955</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.581979</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.501641</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.068918</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.718045</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.707404</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.758738</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>S002</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1.037795</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.566185</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.664801</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.725955</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.581979</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.501641</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1.068918</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.718045</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.707404</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.758738</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S003</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1.037795</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.566185</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.664801</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.725955</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.581979</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.501641</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1.068918</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.718045</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.707404</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.758738</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.254976</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-0.103291</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-0.057809</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-0.058256</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-0.178068</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-0.17888</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.272915</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-0.226751</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.004019</v>
+      </c>
+      <c r="K5" t="n">
+        <v>-0.045984</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>S005</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.254976</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-0.103291</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-0.057809</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-0.058256</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-0.178068</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-0.17888</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.272915</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-0.226751</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.004019</v>
+      </c>
+      <c r="K6" t="n">
+        <v>-0.045984</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>S006</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.254976</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-0.103291</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-0.057809</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-0.058256</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-0.178068</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-0.17888</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.272915</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-0.226751</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.004019</v>
+      </c>
+      <c r="K7" t="n">
+        <v>-0.045984</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>S007</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1.932446</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1.331301</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1.490641</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1.622195</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.450604</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.279379</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1.978636</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1.797813</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1.511272</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1.67842</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>S008</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1.932446</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1.331301</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1.490641</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1.622195</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.450604</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1.279379</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1.978636</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1.797813</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1.511272</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1.67842</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>S009</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>-0.527844</v>
+      </c>
+      <c r="C10" t="n">
+        <v>-0.772767</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-0.780419</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-0.842466</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-0.938115</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-0.859401</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-0.523088</v>
+      </c>
+      <c r="I10" t="n">
+        <v>-1.171548</v>
+      </c>
+      <c r="J10" t="n">
+        <v>-0.699365</v>
+      </c>
+      <c r="K10" t="n">
+        <v>-0.850706</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>S010</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>-0.527844</v>
+      </c>
+      <c r="C11" t="n">
+        <v>-0.772767</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-0.780419</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-0.842466</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-0.938115</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-0.859401</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-0.523088</v>
+      </c>
+      <c r="I11" t="n">
+        <v>-1.171548</v>
+      </c>
+      <c r="J11" t="n">
+        <v>-0.699365</v>
+      </c>
+      <c r="K11" t="n">
+        <v>-0.850706</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>S011</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>-0.527844</v>
+      </c>
+      <c r="C12" t="n">
+        <v>-0.772767</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-0.780419</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-0.842466</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-0.938115</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-0.859401</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-0.523088</v>
+      </c>
+      <c r="I12" t="n">
+        <v>-1.171548</v>
+      </c>
+      <c r="J12" t="n">
+        <v>-0.699365</v>
+      </c>
+      <c r="K12" t="n">
+        <v>-0.850706</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>S012</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>-0.639675</v>
+      </c>
+      <c r="C13" t="n">
+        <v>-0.485848</v>
+      </c>
+      <c r="D13" t="n">
+        <v>-0.986879</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.165804</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-1.155271</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1.182162</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-1.091661</v>
+      </c>
+      <c r="I13" t="n">
+        <v>-1.846402</v>
+      </c>
+      <c r="J13" t="n">
+        <v>-1.503233</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.183936</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>S013</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>-1.087001</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.948743</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-0.883649</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.725955</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1.66776</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-1.151053</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-2.569952</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.313133</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.405953</v>
+      </c>
+      <c r="K14" t="n">
+        <v>-0.390865</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>S014</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.254976</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1.044382</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-1.709489</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-0.058256</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1.559182</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-0.956618</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-0.068229</v>
+      </c>
+      <c r="I15" t="n">
+        <v>-0.631664</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.908371</v>
+      </c>
+      <c r="K15" t="n">
+        <v>-2.115269</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>S015</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>-0.19235</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.757464</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1.284181</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-1.290586</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.147666</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-0.5677489999999999</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.500345</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1.527871</v>
+      </c>
+      <c r="J16" t="n">
+        <v>-1.7042</v>
+      </c>
+      <c r="K16" t="n">
+        <v>-1.195587</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>S016</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>-0.08051899999999999</v>
+      </c>
+      <c r="C17" t="n">
+        <v>-2.111718</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-1.812719</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-0.282316</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.256244</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-0.17888</v>
+      </c>
+      <c r="H17" t="n">
+        <v>-0.523088</v>
+      </c>
+      <c r="I17" t="n">
+        <v>-0.496693</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.30547</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.183936</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>S017</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>-1.310664</v>
+      </c>
+      <c r="C18" t="n">
+        <v>-1.537882</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.871261</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-1.962766</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.581979</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.307207</v>
+      </c>
+      <c r="H18" t="n">
+        <v>-0.750517</v>
+      </c>
+      <c r="I18" t="n">
+        <v>-0.361722</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.506437</v>
+      </c>
+      <c r="K18" t="n">
+        <v>-0.735746</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>S018</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>-0.639675</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.566185</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.561571</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1.174075</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-1.481006</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-0.081663</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.045486</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.853016</v>
+      </c>
+      <c r="J19" t="n">
+        <v>-0.498398</v>
+      </c>
+      <c r="K19" t="n">
+        <v>-1.425507</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>S019</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.5904700000000001</v>
+      </c>
+      <c r="C20" t="n">
+        <v>-1.729161</v>
+      </c>
+      <c r="D20" t="n">
+        <v>-1.090109</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-0.282316</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.907713</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-1.734356</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-0.523088</v>
+      </c>
+      <c r="I20" t="n">
+        <v>-1.036577</v>
+      </c>
+      <c r="J20" t="n">
+        <v>-2.206617</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.183936</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>S020</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>-0.416013</v>
+      </c>
+      <c r="C21" t="n">
+        <v>-0.390209</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.148651</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-1.514646</v>
+      </c>
+      <c r="F21" t="n">
+        <v>-1.698162</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.9877280000000001</v>
+      </c>
+      <c r="H21" t="n">
+        <v>-0.068229</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.9879869999999999</v>
+      </c>
+      <c r="J21" t="n">
+        <v>1.209821</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.183936</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>S021</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>-0.863338</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1.618219</v>
+      </c>
+      <c r="D22" t="n">
+        <v>-0.367499</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-0.730436</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.039088</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.501641</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.614059</v>
+      </c>
+      <c r="I22" t="n">
+        <v>-1.036577</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.707404</v>
+      </c>
+      <c r="K22" t="n">
+        <v>-1.080626</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>S022</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0.702301</v>
+      </c>
+      <c r="C23" t="n">
+        <v>-0.294569</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-0.986879</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.725955</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.147666</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-0.859401</v>
+      </c>
+      <c r="H23" t="n">
+        <v>-0.636802</v>
+      </c>
+      <c r="I23" t="n">
+        <v>-0.361722</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.807887</v>
+      </c>
+      <c r="K23" t="n">
+        <v>1.333539</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>S023</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>-0.304181</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.566185</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1.077721</v>
+      </c>
+      <c r="E24" t="n">
+        <v>-1.178556</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-0.503802</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-1.734356</v>
+      </c>
+      <c r="H24" t="n">
+        <v>-0.068229</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.448103</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.104503</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0.758738</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>S024</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0.366807</v>
+      </c>
+      <c r="C25" t="n">
+        <v>-1.155324</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-0.057809</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1.622195</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-1.698162</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1.765466</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.045486</v>
+      </c>
+      <c r="I25" t="n">
+        <v>-0.631664</v>
+      </c>
+      <c r="J25" t="n">
+        <v>-1.101299</v>
+      </c>
+      <c r="K25" t="n">
+        <v>1.448499</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>S025</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>-2.540809</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.470546</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1.490641</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.165804</v>
+      </c>
+      <c r="F26" t="n">
+        <v>-0.06949</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1.571031</v>
+      </c>
+      <c r="H26" t="n">
+        <v>-1.319091</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.718045</v>
+      </c>
+      <c r="J26" t="n">
+        <v>-1.000815</v>
+      </c>
+      <c r="K26" t="n">
+        <v>-0.275905</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -895,11 +3587,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>class_average</t>
+          <t>class_weighted_average</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>80.40000000000001</v>
+        <v>75.41</v>
       </c>
     </row>
     <row r="3">
@@ -909,7 +3601,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>81</v>
+        <v>74.90000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -939,7 +3631,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -969,7 +3661,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -989,7 +3681,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
@@ -999,7 +3691,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1009,7 +3701,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -1050,7 +3742,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S016</t>
         </is>
       </c>
     </row>
@@ -1062,7 +3754,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S007</t>
         </is>
       </c>
     </row>

</xml_diff>